<commit_message>
:motorcycle::motorcycle: rarefy dataset with 2 chimeras filtering
</commit_message>
<xml_diff>
--- a/data/derived_data/2_RarefyData/Conta_clusters_ITS.xlsx
+++ b/data/derived_data/2_RarefyData/Conta_clusters_ITS.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -119,15 +119,9 @@
     <t xml:space="preserve">Cluster_960</t>
   </si>
   <si>
-    <t xml:space="preserve">Cluster_1002</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cluster_1020</t>
   </si>
   <si>
-    <t xml:space="preserve">Cluster_1251</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cluster_1503</t>
   </si>
   <si>
@@ -137,37 +131,19 @@
     <t xml:space="preserve">Cluster_1739</t>
   </si>
   <si>
-    <t xml:space="preserve">Cluster_2070</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cluster_2117</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_2476</t>
   </si>
   <si>
-    <t xml:space="preserve">Cluster_3100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cluster_3166</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cluster_3205</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cluster_3378</t>
   </si>
   <si>
-    <t xml:space="preserve">Cluster_3466</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cluster_3822</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_4031</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cluster_4128</t>
   </si>
   <si>
     <t xml:space="preserve">Cluster_4156</t>
@@ -999,7 +975,7 @@
         <v>14</v>
       </c>
       <c r="H19" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20">
@@ -1025,7 +1001,7 @@
         <v>14</v>
       </c>
       <c r="H20" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21">
@@ -1051,7 +1027,7 @@
         <v>14</v>
       </c>
       <c r="H21" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22">
@@ -1077,7 +1053,7 @@
         <v>14</v>
       </c>
       <c r="H22" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="23">
@@ -1155,7 +1131,7 @@
         <v>14</v>
       </c>
       <c r="H25" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
     </row>
     <row r="26">
@@ -1181,7 +1157,7 @@
         <v>14</v>
       </c>
       <c r="H26" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="27">
@@ -1233,7 +1209,7 @@
         <v>14</v>
       </c>
       <c r="H28" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="29">
@@ -1285,7 +1261,7 @@
         <v>14</v>
       </c>
       <c r="H30" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="31">
@@ -1311,214 +1287,6 @@
         <v>14</v>
       </c>
       <c r="H31" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="s">
-        <v>48</v>
-      </c>
-      <c r="B32" t="s">
-        <v>9</v>
-      </c>
-      <c r="C32" t="s">
-        <v>10</v>
-      </c>
-      <c r="D32" t="s">
-        <v>11</v>
-      </c>
-      <c r="E32" t="s">
-        <v>12</v>
-      </c>
-      <c r="F32" t="s">
-        <v>13</v>
-      </c>
-      <c r="G32" t="s">
-        <v>14</v>
-      </c>
-      <c r="H32" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="s">
-        <v>49</v>
-      </c>
-      <c r="B33" t="s">
-        <v>9</v>
-      </c>
-      <c r="C33" t="s">
-        <v>10</v>
-      </c>
-      <c r="D33" t="s">
-        <v>11</v>
-      </c>
-      <c r="E33" t="s">
-        <v>12</v>
-      </c>
-      <c r="F33" t="s">
-        <v>13</v>
-      </c>
-      <c r="G33" t="s">
-        <v>14</v>
-      </c>
-      <c r="H33" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="s">
-        <v>50</v>
-      </c>
-      <c r="B34" t="s">
-        <v>9</v>
-      </c>
-      <c r="C34" t="s">
-        <v>10</v>
-      </c>
-      <c r="D34" t="s">
-        <v>11</v>
-      </c>
-      <c r="E34" t="s">
-        <v>12</v>
-      </c>
-      <c r="F34" t="s">
-        <v>13</v>
-      </c>
-      <c r="G34" t="s">
-        <v>14</v>
-      </c>
-      <c r="H34" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="s">
-        <v>51</v>
-      </c>
-      <c r="B35" t="s">
-        <v>9</v>
-      </c>
-      <c r="C35" t="s">
-        <v>10</v>
-      </c>
-      <c r="D35" t="s">
-        <v>11</v>
-      </c>
-      <c r="E35" t="s">
-        <v>12</v>
-      </c>
-      <c r="F35" t="s">
-        <v>13</v>
-      </c>
-      <c r="G35" t="s">
-        <v>14</v>
-      </c>
-      <c r="H35" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="s">
-        <v>52</v>
-      </c>
-      <c r="B36" t="s">
-        <v>9</v>
-      </c>
-      <c r="C36" t="s">
-        <v>10</v>
-      </c>
-      <c r="D36" t="s">
-        <v>11</v>
-      </c>
-      <c r="E36" t="s">
-        <v>12</v>
-      </c>
-      <c r="F36" t="s">
-        <v>13</v>
-      </c>
-      <c r="G36" t="s">
-        <v>14</v>
-      </c>
-      <c r="H36" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="s">
-        <v>53</v>
-      </c>
-      <c r="B37" t="s">
-        <v>9</v>
-      </c>
-      <c r="C37" t="s">
-        <v>10</v>
-      </c>
-      <c r="D37" t="s">
-        <v>11</v>
-      </c>
-      <c r="E37" t="s">
-        <v>12</v>
-      </c>
-      <c r="F37" t="s">
-        <v>13</v>
-      </c>
-      <c r="G37" t="s">
-        <v>14</v>
-      </c>
-      <c r="H37" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="s">
-        <v>54</v>
-      </c>
-      <c r="B38" t="s">
-        <v>9</v>
-      </c>
-      <c r="C38" t="s">
-        <v>10</v>
-      </c>
-      <c r="D38" t="s">
-        <v>11</v>
-      </c>
-      <c r="E38" t="s">
-        <v>12</v>
-      </c>
-      <c r="F38" t="s">
-        <v>13</v>
-      </c>
-      <c r="G38" t="s">
-        <v>14</v>
-      </c>
-      <c r="H38" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="s">
-        <v>55</v>
-      </c>
-      <c r="B39" t="s">
-        <v>9</v>
-      </c>
-      <c r="C39" t="s">
-        <v>10</v>
-      </c>
-      <c r="D39" t="s">
-        <v>11</v>
-      </c>
-      <c r="E39" t="s">
-        <v>12</v>
-      </c>
-      <c r="F39" t="s">
-        <v>13</v>
-      </c>
-      <c r="G39" t="s">
-        <v>14</v>
-      </c>
-      <c r="H39" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>